<commit_message>
renombrar archivo de práctica: agregar formato condicional con función SI
</commit_message>
<xml_diff>
--- a/practicas/archivos_practica/excel-base-01.xlsx
+++ b/practicas/archivos_practica/excel-base-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Optalvis\Downloads\practicas-excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\vanilla\vanilla-blog-excel\practicas\archivos_practica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69B9B37D-E2F9-4482-9A6E-7CF11701D096}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78E1E188-3550-4E2E-A444-8E0483819BEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{39DFF5B5-6AF6-4AAE-B7FC-6E73DD60808C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{39DFF5B5-6AF6-4AAE-B7FC-6E73DD60808C}"/>
   </bookViews>
   <sheets>
     <sheet name="Ejercicio 1" sheetId="1" r:id="rId1"/>
@@ -123,7 +123,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="_ &quot;S/&quot;* #,##0.00_ ;_ &quot;S/&quot;* \-#,##0.00_ ;_ &quot;S/&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ &quot;S/&quot;* #,##0.00_ ;_ &quot;S/&quot;* \-#,##0.00_ ;_ &quot;S/&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -224,18 +224,16 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -767,12 +765,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A068A630-A51D-4CED-B0BC-E3D1F1B3B0BD}" name="Tabla1" displayName="Tabla1" ref="A1:C6" totalsRowShown="0" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A068A630-A51D-4CED-B0BC-E3D1F1B3B0BD}" name="Tabla1" displayName="Tabla1" ref="A1:C6" totalsRowShown="0" dataDxfId="3">
   <autoFilter ref="A1:C6" xr:uid="{A068A630-A51D-4CED-B0BC-E3D1F1B3B0BD}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{74AF555B-7899-4CB4-9849-1B63CBC2483B}" name="Nº" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{E1B8A236-9863-4F9A-BDFB-EDE4DAE06F3B}" name="PREGUNTA" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{2DFFF31E-3C82-4FED-B031-0893169A6C79}" name="RSEPUESTA" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{74AF555B-7899-4CB4-9849-1B63CBC2483B}" name="Nº" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{E1B8A236-9863-4F9A-BDFB-EDE4DAE06F3B}" name="PREGUNTA" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{2DFFF31E-3C82-4FED-B031-0893169A6C79}" name="RSEPUESTA" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1075,7 +1073,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB091369-D3F2-447A-98CD-501E4A75C7CB}">
-  <dimension ref="B2:F11"/>
+  <dimension ref="B2:F10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4.140625" customWidth="1"/>
@@ -1084,135 +1082,131 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="4" t="s">
+      <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
     </row>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="4" t="s">
+      <c r="B3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B4" s="4" t="s">
+      <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4">
         <v>26250</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4">
         <v>74121</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4">
         <v>63742</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4">
         <v>25745</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
+      <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5">
         <v>92696</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5">
         <v>18104</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5">
         <v>94013</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5">
         <v>12602</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B6" s="4" t="s">
+      <c r="B6" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6">
         <v>85869</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6">
         <v>66098</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6">
         <v>45807</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B7" s="4" t="s">
+      <c r="B7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7">
         <v>24819</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7">
         <v>45549</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E7">
         <v>56739</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7">
         <v>66271</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
+      <c r="B8" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8">
         <v>74740</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8">
         <v>58686</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" t="s">
         <v>18</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8">
         <v>54468</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B9" s="4" t="s">
+      <c r="B9" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9">
         <v>96473</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9">
         <v>52119</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9">
         <v>84366</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F9">
         <v>11001</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="5" t="s">
+      <c r="B10" t="s">
         <v>17</v>
       </c>
       <c r="C10">
@@ -1227,9 +1221,6 @@
       <c r="F10">
         <v>36616</v>
       </c>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1255,10 +1246,10 @@
       <c r="J2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="L2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="N2" s="4" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1294,8 +1285,8 @@
     </row>
     <row r="9" spans="10:14" x14ac:dyDescent="0.25">
       <c r="J9" s="3"/>
-      <c r="L9" s="7"/>
-      <c r="N9" s="7"/>
+      <c r="L9" s="5"/>
+      <c r="N9" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1310,7 +1301,7 @@
   <cols>
     <col min="2" max="2" width="69.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.7109375" customWidth="1"/>
-    <col min="7" max="7" width="0" style="8" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="0" style="6" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1323,75 +1314,72 @@
       <c r="C1" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="7" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="11"/>
-      <c r="E2" s="10">
-        <f>SUM(G2:G6)*20</f>
-        <v>0</v>
-      </c>
-      <c r="G2" s="8">
+      <c r="C2" s="9"/>
+      <c r="E2" s="8"/>
+      <c r="G2" s="6">
         <f>IF(Tabla1[[#This Row],[RSEPUESTA]]=94013,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11">
+      <c r="A3" s="9">
         <v>2</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="G3" s="8">
+      <c r="C3" s="9"/>
+      <c r="G3" s="6">
         <f>IF(Tabla1[[#This Row],[RSEPUESTA]]=1411414,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="11">
+      <c r="A4" s="9">
         <v>3</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="11"/>
-      <c r="G4" s="8">
+      <c r="C4" s="9"/>
+      <c r="G4" s="6">
         <f>IF(Tabla1[[#This Row],[RSEPUESTA]]=TRUE,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="11">
+      <c r="A5" s="9">
         <v>4</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="G5" s="8">
+      <c r="C5" s="9"/>
+      <c r="G5" s="6">
         <f>IF(Tabla1[[#This Row],[RSEPUESTA]]=11001,1,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11">
+      <c r="A6" s="9">
         <v>5</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="11"/>
-      <c r="G6" s="8">
+      <c r="C6" s="9"/>
+      <c r="G6" s="6">
         <f>IF(Tabla1[[#This Row],[RSEPUESTA]]=94013,1,0)</f>
         <v>0</v>
       </c>

</xml_diff>